<commit_message>
Upload latest version of XFSU Mapping
</commit_message>
<xml_diff>
--- a/Documentation_website/docs/Orchestration/assets/Orchestration-1.2.0-XFSU-6.0.0-mapping.xlsx
+++ b/Documentation_website/docs/Orchestration/assets/Orchestration-1.2.0-XFSU-6.0.0-mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iataonline-my.sharepoint.com/personal/lambertc_iata_org/Documents/ONE Record/31 CXML mapping/Ochestration 1.2.0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="671" documentId="8_{B25369B4-3DC5-4B93-B3E9-B78377898FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A30F4D7C-B7D6-40F7-A7BA-87F98611322B}"/>
+  <xr:revisionPtr revIDLastSave="824" documentId="8_{B25369B4-3DC5-4B93-B3E9-B78377898FF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC021D46-28D2-4AB0-BF5A-5108B483C5C5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{05E5835E-21B0-44A2-A276-1010F8666971}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="332">
   <si>
     <t>1:n</t>
   </si>
@@ -773,12 +773,6 @@
     <t>Refer to Waybill#waybillType in correlation with UN/EDIFACT codes</t>
   </si>
   <si>
-    <t>Either drill drown to Booking with TransportLegs or refer to TransportMovements linked to Pieces/ULDs</t>
-  </si>
-  <si>
-    <t>Event is either on Shipment or Pieces depending on the scenario</t>
-  </si>
-  <si>
     <t>Waybill#serviceCode</t>
   </si>
   <si>
@@ -791,15 +785,6 @@
     <t>Use the MovementType with appropriate movementTimeType and movementMilestone</t>
   </si>
   <si>
-    <t>partyRole = AIR ?</t>
-  </si>
-  <si>
-    <t>N/A for OSI/SSR - Waybill#shipment -&gt; Shipment#pieces -&gt;Piece#specialHandlingCodes (SPH)</t>
-  </si>
-  <si>
-    <t>Waybill#shipment -&gt; Shipment#textualHandlingInstructions (OSI, SSR) - Retrieve from Code List for SPH</t>
-  </si>
-  <si>
     <t>Shipment OR Piece level CustomsInformation depending on availability</t>
   </si>
   <si>
@@ -818,18 +803,9 @@
     <t>House Waybill details</t>
   </si>
   <si>
-    <t>Is it used?</t>
-  </si>
-  <si>
     <t>Waybill object with waybillType = HOUSE</t>
   </si>
   <si>
-    <t>Is info at line item level?</t>
-  </si>
-  <si>
-    <t>waybill#shipment -&gt; Shipment#totalGrossWeight</t>
-  </si>
-  <si>
     <t>No prefix required if House</t>
   </si>
   <si>
@@ -842,114 +818,18 @@
     <t>The couting depends if this is a part shipment or not</t>
   </si>
   <si>
-    <t>Linked to distribution, how is it relevant to status code? Optional, I suggest to leave it out in the mapping.</t>
-  </si>
-  <si>
-    <t>Do we need an additional property? Can it be used with locationType?</t>
-  </si>
-  <si>
     <t>Would propose a subtype of LogisticsEvent for FIW/FOW with handoverLocation</t>
   </si>
   <si>
     <t>Geolocation specific to FIW/FOW, recommend usage of Location specific for FIW/FOW</t>
   </si>
   <si>
-    <t>LogisticsEvent#eventDate</t>
-  </si>
-  <si>
-    <t>LogisticsEvent#eventTimeType</t>
-  </si>
-  <si>
-    <t>Exact path depends on the object used for the LogisticsEvent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LogisticsEvent#involvedParties -&gt; Party#partyDetails -&gt; Company#name </t>
-  </si>
-  <si>
     <t>PartyRole = NI</t>
   </si>
   <si>
     <t>PartyRole = ST (Ship To)</t>
   </si>
   <si>
-    <t>LogisticsEvent#recordingOrganization</t>
-  </si>
-  <si>
-    <t>Not in 1R for the moment</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt;Piece#involvedInActions -&gt; Loading#servedActivity -&gt; TransportMovement#transportIdentifier</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt;Piece#involvedInActions -&gt; Loading#servedActivity -&gt; Transportmovement#transportOrganization -&gt; Carrier#airlineCode</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt;Piece#involvedInActions -&gt; Loading#servedActivity -&gt; Transportmovement#transportMeans -&gt; TransportMeans#vehicleType</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt;Piece#involvedInActions -&gt; Loading#servedActivity -&gt; TransportMovement#movementTimes -&gt; MovementTime#movementTimestamp</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt;Piece#involvedInActions -&gt; Loading#servedActivity -&gt; TransportMovement#movementTimes -&gt; MovementTime#movementTimeType</t>
-  </si>
-  <si>
-    <t>Shipment#involvedParties -&gt; Party#partyDetails -&gt; Carrier#airlineCode</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#events -&gt; LogisticsEvent#eventLocation -&gt; Location#locationsCodes -&gt; CodeListElement#code</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#events -&gt; LogisticsEvent#eventLocation -&gt; Location#locationName</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#events -&gt; LogisticsEvent#eventLocation -&gt; Location#locationType</t>
-  </si>
-  <si>
-    <t>Shipment#customsInformation -&gt; CustomsInformation#contentCode</t>
-  </si>
-  <si>
-    <t>Shipment#customsInformation -&gt; CustomsInformation#note</t>
-  </si>
-  <si>
-    <t>Shipment#customsInformation -&gt; CustomsInformation#subjectCode</t>
-  </si>
-  <si>
-    <t>Shipment#customsInformation -&gt; CustomsInformation#countryCode</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#involvedInActions -&gt; UnitComposition#onLoadingUnit -&gt; ULD#uldSerialNumber</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#involvedInActions -&gt; UnitComposition#onLoadingUnit -&gt; ULD#uldTypeCode</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#involvedInActions -&gt; UnitComposition#onLoadingUnit -&gt; ULD#loadingIndicator</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#involvedInActions -&gt; UnitComposition#onLoadingUnit -&gt; ULD#serviceabilityCode</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#involvedInActions -&gt; UnitComposition#onLoadingUnit -&gt; ULD#ownerCode</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#involvedInActions -&gt; UnitComposition#onLoadingUnit -&gt; LoadingUnit# ?</t>
-  </si>
-  <si>
-    <t>Shipment#waybill -&gt; Waybill#waybillNumber</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#events -&gt; LogisticsEvent#eventCode (Or Shipment#events)</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#grossWeight or Shipment#totalGrossWeight</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Piece#dimensions or Shipment#totalDimensions</t>
-  </si>
-  <si>
-    <t>Shipment#pieces -&gt; Count all connected Pieces if identified, otherwise ?</t>
-  </si>
-  <si>
     <t>Shipment#externalReferences</t>
   </si>
   <si>
@@ -968,15 +848,9 @@
     <t>Count all connected Pieces</t>
   </si>
   <si>
-    <t>LogisticsEvent#partialEventIndicator</t>
-  </si>
-  <si>
     <t>Shipment#pieces</t>
   </si>
   <si>
-    <t>StatusUpdateEvent#recordedPieceCount</t>
-  </si>
-  <si>
     <t>Waybill#waybilPrefix+'-'+Waybill#waybilNumber</t>
   </si>
   <si>
@@ -996,6 +870,171 @@
   </si>
   <si>
     <t>Only T and P are used in (X)FSU, True = P</t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#partialEventIndicator</t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#eventCode</t>
+  </si>
+  <si>
+    <t>IATA Airport code or UNLOCODE. The Routing must be entered if: places of departure and destination are within the same territory and one or more agreed stopping places being within the territory of another State then an indication of at least one such stopping place must be indicated.</t>
+  </si>
+  <si>
+    <t>To be checked if there is usage of that fields</t>
+  </si>
+  <si>
+    <t>Mapping will depend on the scenario: Partial or not</t>
+  </si>
+  <si>
+    <t>Shipment#pieces -&gt; Piece#grossWeight or Shipment#totalGrossWeight
+StatusUpdateEvent#recordedWeight if StatusUpdateEvent#partialEventIndicator = True</t>
+  </si>
+  <si>
+    <t>Shipment#pieces -&gt; Piece#dimensions or Shipment#Shipment#totalVolume
+StatusUpdateEvent#recordedVolumet if StatusUpdateEvent#partialEventIndicator = True</t>
+  </si>
+  <si>
+    <t>Shipment#pieces -&gt; Count all connected Pieces
+StatusUpdateEvent#recordedPieceCount if StatusUpdateEvent#partialEventIndicator = True</t>
+  </si>
+  <si>
+    <t>Based on StatusUpdateEvent#partialEventIndicator value</t>
+  </si>
+  <si>
+    <t>TransportMovement#transportIdentifier</t>
+  </si>
+  <si>
+    <t>Transportmovement#transportOrganization</t>
+  </si>
+  <si>
+    <t>Carrier#airlineCode</t>
+  </si>
+  <si>
+    <t>TransportMeans#vehicleType</t>
+  </si>
+  <si>
+    <t>Transportmovement#transportMeans</t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#transportMovementReference</t>
+  </si>
+  <si>
+    <t>MovementTime#movementTimestamp</t>
+  </si>
+  <si>
+    <t>TransportMovement#movementTimes</t>
+  </si>
+  <si>
+    <t>MovementTime#movementType</t>
+  </si>
+  <si>
+    <t>Party#partyDetails</t>
+  </si>
+  <si>
+    <t>Shipment#involvedParties</t>
+  </si>
+  <si>
+    <t>Location#locationsCodes</t>
+  </si>
+  <si>
+    <t>CodeListElement#code</t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#eventLocation</t>
+  </si>
+  <si>
+    <t>Location#locationName</t>
+  </si>
+  <si>
+    <t>Location#locationType</t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#eventDate</t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#eventTimeType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company#name </t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#recordingOrganization</t>
+  </si>
+  <si>
+    <t>StatusUpdateEvent#transferredFrom</t>
+  </si>
+  <si>
+    <t>partyRole = CA</t>
+  </si>
+  <si>
+    <t>RoleCode = CA by default</t>
+  </si>
+  <si>
+    <t>Company#name</t>
+  </si>
+  <si>
+    <t>Shipment#textualHandlingInstructions (OSI, SSR) - Retrieve from Code List for SPH</t>
+  </si>
+  <si>
+    <t>Waybill#shipment</t>
+  </si>
+  <si>
+    <t>N/A for OSI/SSR</t>
+  </si>
+  <si>
+    <t>Piece#specialHandlingCodes (SPH)</t>
+  </si>
+  <si>
+    <t>CustomsInformation#contentCode</t>
+  </si>
+  <si>
+    <t>CustomsInformation#subjectCode</t>
+  </si>
+  <si>
+    <t>CustomsInformation#countryCode</t>
+  </si>
+  <si>
+    <t>CustomsInformation#otherCustomsInformation</t>
+  </si>
+  <si>
+    <t>Shipment#customsInformation</t>
+  </si>
+  <si>
+    <t>Piece#involvedInActions</t>
+  </si>
+  <si>
+    <t>UnitComposition#onLoadingUnit</t>
+  </si>
+  <si>
+    <t>ULD#uldSerialNumber</t>
+  </si>
+  <si>
+    <t>ULD#uldTypeCode</t>
+  </si>
+  <si>
+    <t>ULD#loadingIndicator</t>
+  </si>
+  <si>
+    <t>ULD#serviceabilityCode</t>
+  </si>
+  <si>
+    <t>ULD#ownerCode</t>
+  </si>
+  <si>
+    <t>LoadingUnit# ?</t>
+  </si>
+  <si>
+    <t>waybill#shipment</t>
+  </si>
+  <si>
+    <t>Waybill#waybillNumber</t>
+  </si>
+  <si>
+    <t>Is it used, shall we use the same as ULD ?</t>
+  </si>
+  <si>
+    <t>Refer to House level details but no evidence of usage</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1090,6 +1129,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1404,17 +1447,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{316EC749-09E5-4BD0-84BE-791558487EE8}">
-  <dimension ref="A1:N161"/>
+  <dimension ref="A1:P160"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="1" customWidth="1"/>
     <col min="2" max="6" width="5" customWidth="1"/>
-    <col min="7" max="7" width="44.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="9.140625" style="3"/>
     <col min="11" max="11" width="28.5703125" style="8" customWidth="1"/>
     <col min="12" max="12" width="36.7109375" style="10" customWidth="1"/>
-    <col min="13" max="13" width="42.28515625" customWidth="1"/>
+    <col min="13" max="13" width="53.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -1475,10 +1518,10 @@
         <v>144</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>306</v>
+        <v>266</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>307</v>
+        <v>267</v>
       </c>
       <c r="N3" s="1"/>
     </row>
@@ -1766,10 +1809,10 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I24" s="3" t="s">
         <v>135</v>
@@ -1778,31 +1821,39 @@
         <v>2</v>
       </c>
       <c r="K24" s="7"/>
+      <c r="M24" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H25" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K25" s="7"/>
+        <v>4</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>145</v>
+      </c>
       <c r="M25" t="s">
-        <v>305</v>
+        <v>270</v>
+      </c>
+      <c r="N25" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H26" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>127</v>
@@ -1810,22 +1861,22 @@
       <c r="J26" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K26" s="7" t="s">
-        <v>145</v>
+      <c r="K26" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="L26" s="10" t="s">
+        <v>259</v>
       </c>
       <c r="M26" t="s">
-        <v>311</v>
-      </c>
-      <c r="N26" t="s">
-        <v>308</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H27" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>127</v>
@@ -1834,21 +1885,21 @@
         <v>4</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="L27" s="10" t="s">
-        <v>267</v>
+        <v>149</v>
       </c>
       <c r="M27" t="s">
-        <v>312</v>
+        <v>270</v>
+      </c>
+      <c r="N27" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H28" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I28" s="3" t="s">
         <v>127</v>
@@ -1857,315 +1908,310 @@
         <v>4</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>149</v>
+        <v>168</v>
+      </c>
+      <c r="L28" s="10" t="s">
+        <v>277</v>
       </c>
       <c r="M28" t="s">
-        <v>311</v>
-      </c>
-      <c r="N28" t="s">
-        <v>309</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B29" t="s">
-        <v>25</v>
-      </c>
-      <c r="H29" t="s">
-        <v>150</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J29" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K29" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="L29" s="11" t="s">
-        <v>319</v>
-      </c>
-      <c r="M29" t="s">
-        <v>310</v>
+      <c r="B29" s="1" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="1" t="s">
-        <v>99</v>
+      <c r="B30" s="1"/>
+      <c r="C30" t="s">
+        <v>6</v>
+      </c>
+      <c r="H30" t="s">
+        <v>151</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="M30" t="s">
+        <v>272</v>
+      </c>
+      <c r="N30" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
       <c r="C31" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H31" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="L31" s="10" t="s">
+        <v>243</v>
       </c>
       <c r="M31" t="s">
-        <v>314</v>
-      </c>
-      <c r="N31" t="s">
-        <v>313</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
       <c r="C32" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="H32" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K32" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="L32" s="10" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="M32" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="33" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B33" s="1"/>
-      <c r="C33" t="s">
-        <v>26</v>
-      </c>
-      <c r="H33" t="s">
-        <v>154</v>
-      </c>
-      <c r="I33" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J33" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K33" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="L33" s="10" t="s">
-        <v>244</v>
-      </c>
-      <c r="M33" t="s">
-        <v>235</v>
+      <c r="B33" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="34" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
-        <v>27</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B35" s="1" t="s">
-        <v>100</v>
+      <c r="B35" s="1"/>
+      <c r="C35" t="s">
+        <v>6</v>
+      </c>
+      <c r="H35" t="s">
+        <v>156</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="M35" t="s">
+        <v>272</v>
+      </c>
+      <c r="N35" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="36" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
       <c r="C36" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H36" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K36" s="8" t="s">
-        <v>157</v>
+        <v>2</v>
       </c>
       <c r="M36" t="s">
-        <v>314</v>
+        <v>272</v>
       </c>
       <c r="N36" t="s">
-        <v>315</v>
+        <v>274</v>
       </c>
     </row>
     <row r="37" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B37" s="1"/>
-      <c r="C37" t="s">
-        <v>7</v>
-      </c>
-      <c r="H37" t="s">
-        <v>158</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J37" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="M37" t="s">
-        <v>314</v>
-      </c>
-      <c r="N37" t="s">
-        <v>316</v>
+      <c r="B37" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
-        <v>28</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B39" s="1" t="s">
-        <v>101</v>
+      <c r="B39" s="1"/>
+      <c r="C39" t="s">
+        <v>6</v>
+      </c>
+      <c r="H39" t="s">
+        <v>159</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="M39" t="s">
+        <v>272</v>
+      </c>
+      <c r="N39" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
       <c r="C40" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H40" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K40" s="8" t="s">
-        <v>157</v>
+        <v>2</v>
       </c>
       <c r="M40" t="s">
-        <v>314</v>
+        <v>272</v>
       </c>
       <c r="N40" t="s">
-        <v>317</v>
+        <v>276</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B41" s="1"/>
-      <c r="C41" t="s">
-        <v>7</v>
-      </c>
-      <c r="H41" t="s">
-        <v>160</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J41" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="M41" t="s">
-        <v>314</v>
-      </c>
-      <c r="N41" t="s">
-        <v>318</v>
+      <c r="B41" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B42" s="1" t="s">
-        <v>29</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B43" s="1" t="s">
-        <v>102</v>
+      <c r="B43" s="1"/>
+      <c r="C43" t="s">
+        <v>6</v>
+      </c>
+      <c r="H43" t="s">
+        <v>161</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J43" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="K43" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="L43" s="10" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
       <c r="C44" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H44" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I44" s="3" t="s">
         <v>135</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="K44" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="L44" s="11" t="s">
-        <v>245</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B45" s="1"/>
-      <c r="C45" t="s">
-        <v>7</v>
-      </c>
-      <c r="H45" t="s">
-        <v>162</v>
-      </c>
-      <c r="I45" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>2</v>
+      <c r="B45" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
     </row>
     <row r="47" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="1" t="s">
-        <v>103</v>
+      <c r="B47" s="1"/>
+      <c r="C47" t="s">
+        <v>31</v>
+      </c>
+      <c r="H47" t="s">
+        <v>163</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K47" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="M47" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
-      <c r="C48" t="s">
-        <v>31</v>
-      </c>
-      <c r="H48" t="s">
-        <v>163</v>
-      </c>
-      <c r="I48" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K48" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="L48" s="11" t="s">
-        <v>246</v>
-      </c>
-      <c r="M48" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="C48" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="L48" s="10" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="49" spans="2:15" ht="60" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
-      <c r="C49" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D49" t="s">
+        <v>20</v>
+      </c>
+      <c r="H49" t="s">
+        <v>141</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M49" s="12" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="50" spans="2:15" ht="60" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
       <c r="D50" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="H50" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="I50" s="3" t="s">
         <v>135</v>
@@ -2173,17 +2219,20 @@
       <c r="J50" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M50" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K50" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="M50" s="12" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="51" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
       <c r="D51" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H51" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I51" s="3" t="s">
         <v>135</v>
@@ -2192,43 +2241,40 @@
         <v>2</v>
       </c>
       <c r="K51" s="8" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="M51" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="52" spans="2:15" ht="45" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
       <c r="D52" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="H52" t="s">
-        <v>166</v>
+        <v>146</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K52" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="L52" s="11" t="s">
-        <v>268</v>
-      </c>
-      <c r="M52" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+      <c r="M52" s="12" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="53" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
       <c r="D53" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H53" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="I53" s="3" t="s">
         <v>127</v>
@@ -2237,158 +2283,173 @@
         <v>4</v>
       </c>
       <c r="K53" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="L53" s="11"/>
-      <c r="M53" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+      <c r="M53" s="12" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="54" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
       <c r="D54" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="H54" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="I54" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J54" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K54" s="8" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+      <c r="M54" s="12" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="55" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
-      <c r="D55" t="s">
-        <v>34</v>
-      </c>
-      <c r="H55" t="s">
-        <v>170</v>
-      </c>
-      <c r="I55" s="3" t="s">
+      <c r="D55" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="56" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" t="s">
+        <v>6</v>
+      </c>
+      <c r="H56" t="s">
+        <v>172</v>
+      </c>
+      <c r="I56" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="J55" s="4" t="s">
+      <c r="J56" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="K55" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="L55" s="11" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B56" s="1"/>
-      <c r="D56" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="M56" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="57" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
-      <c r="D57" s="1"/>
-      <c r="E57" t="s">
-        <v>6</v>
-      </c>
-      <c r="H57" t="s">
-        <v>172</v>
-      </c>
-      <c r="I57" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J57" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="M57" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D57" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="58" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
       <c r="D58" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="59" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
-      <c r="D59" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D59" s="1"/>
+      <c r="E59" t="s">
+        <v>36</v>
+      </c>
+      <c r="H59" t="s">
+        <v>173</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J59" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K59" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="M59" t="s">
+        <v>272</v>
+      </c>
+      <c r="N59" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="60" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
-      <c r="D60" s="1"/>
-      <c r="E60" t="s">
-        <v>36</v>
-      </c>
-      <c r="H60" t="s">
-        <v>173</v>
-      </c>
-      <c r="I60" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J60" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K60" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="M60" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D60" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="61" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
       <c r="D61" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="62" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
-      <c r="D62" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E62" t="s">
+        <v>6</v>
+      </c>
+      <c r="H62" t="s">
+        <v>175</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J62" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K62" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="M62" t="s">
+        <v>292</v>
+      </c>
+      <c r="N62" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="63" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
-      <c r="E63" t="s">
-        <v>6</v>
-      </c>
-      <c r="H63" t="s">
-        <v>175</v>
-      </c>
-      <c r="I63" s="3" t="s">
+      <c r="E63" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="64" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B64" s="1"/>
+      <c r="E64" s="1"/>
+      <c r="F64" t="s">
+        <v>7</v>
+      </c>
+      <c r="H64" t="s">
+        <v>177</v>
+      </c>
+      <c r="I64" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="J63" s="4" t="s">
+      <c r="J64" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="K63" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="M63" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B64" s="1"/>
-      <c r="E64" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="65" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="K64" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="M64" t="s">
+        <v>292</v>
+      </c>
+      <c r="N64" t="s">
+        <v>288</v>
+      </c>
+      <c r="O64" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="65" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="H65" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I65" s="3" t="s">
         <v>135</v>
@@ -2396,86 +2457,107 @@
       <c r="J65" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="K65" s="8" t="s">
-        <v>178</v>
-      </c>
       <c r="M65" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="66" spans="2:13" x14ac:dyDescent="0.25">
+        <v>292</v>
+      </c>
+      <c r="N65" t="s">
+        <v>291</v>
+      </c>
+      <c r="O65" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="66" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
-      <c r="E66" s="1"/>
-      <c r="F66" t="s">
-        <v>38</v>
-      </c>
-      <c r="H66" t="s">
-        <v>179</v>
-      </c>
-      <c r="I66" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J66" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="M66" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="67" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E66" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="67" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
       <c r="E67" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="68" spans="2:13" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="68" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
-      <c r="E68" s="1" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="69" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E68" s="1"/>
+      <c r="F68" t="s">
+        <v>40</v>
+      </c>
+      <c r="H68" t="s">
+        <v>180</v>
+      </c>
+      <c r="I68" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J68" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="L68" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="M68" t="s">
+        <v>292</v>
+      </c>
+      <c r="N68" t="s">
+        <v>294</v>
+      </c>
+      <c r="O68" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="69" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
-      <c r="E69" s="1"/>
-      <c r="F69" t="s">
-        <v>40</v>
-      </c>
-      <c r="H69" t="s">
-        <v>180</v>
-      </c>
-      <c r="I69" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J69" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="L69" s="10" t="s">
-        <v>249</v>
-      </c>
-      <c r="M69" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="70" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E69" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="70" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
       <c r="E70" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="71" spans="2:13" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="71" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
-      <c r="E71" s="1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="72" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E71" s="1"/>
+      <c r="F71" t="s">
+        <v>42</v>
+      </c>
+      <c r="H71" t="s">
+        <v>181</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J71" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L71" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="M71" t="s">
+        <v>292</v>
+      </c>
+      <c r="N71" t="s">
+        <v>294</v>
+      </c>
+      <c r="O71" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="72" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
       <c r="E72" s="1"/>
       <c r="F72" t="s">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="G72" t="s">
+        <v>246</v>
       </c>
       <c r="H72" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I72" s="3" t="s">
         <v>127</v>
@@ -2483,58 +2565,64 @@
       <c r="J72" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="L72" s="10" t="s">
-        <v>250</v>
+      <c r="K72" s="8" t="s">
+        <v>183</v>
       </c>
       <c r="M72" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="73" spans="2:13" x14ac:dyDescent="0.25">
+        <v>292</v>
+      </c>
+      <c r="N72" t="s">
+        <v>294</v>
+      </c>
+      <c r="O72" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="73" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
-      <c r="E73" s="1"/>
-      <c r="F73" t="s">
-        <v>43</v>
-      </c>
-      <c r="G73" t="s">
-        <v>248</v>
-      </c>
-      <c r="H73" t="s">
-        <v>182</v>
-      </c>
-      <c r="I73" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J73" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K73" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="M73" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="74" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E73" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="74" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
       <c r="E74" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="75" spans="2:13" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="75" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
-      <c r="E75" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="76" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E75" s="1"/>
+      <c r="F75" t="s">
+        <v>45</v>
+      </c>
+      <c r="H75" t="s">
+        <v>181</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="M75" t="s">
+        <v>292</v>
+      </c>
+      <c r="N75" t="s">
+        <v>294</v>
+      </c>
+      <c r="O75" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="76" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
       <c r="E76" s="1"/>
       <c r="F76" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H76" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I76" s="3" t="s">
         <v>127</v>
@@ -2542,130 +2630,157 @@
       <c r="J76" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="K76" s="8" t="s">
+        <v>183</v>
+      </c>
       <c r="M76" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="77" spans="2:13" x14ac:dyDescent="0.25">
+        <v>292</v>
+      </c>
+      <c r="N76" t="s">
+        <v>294</v>
+      </c>
+      <c r="O76" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="77" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
-      <c r="E77" s="1"/>
-      <c r="F77" t="s">
-        <v>46</v>
-      </c>
-      <c r="H77" t="s">
-        <v>182</v>
-      </c>
-      <c r="I77" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J77" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K77" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="M77" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="78" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E77" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="78" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
       <c r="E78" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="79" spans="2:13" x14ac:dyDescent="0.25">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="79" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
-      <c r="E79" s="1" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="80" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E79" s="1"/>
+      <c r="F79" t="s">
+        <v>48</v>
+      </c>
+      <c r="H79" t="s">
+        <v>184</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J79" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K79" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="L79" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="M79" t="s">
+        <v>297</v>
+      </c>
+      <c r="N79" t="s">
+        <v>296</v>
+      </c>
+      <c r="O79" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="80" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
-      <c r="E80" s="1"/>
-      <c r="F80" t="s">
-        <v>48</v>
-      </c>
-      <c r="H80" t="s">
-        <v>184</v>
-      </c>
-      <c r="I80" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J80" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K80" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="L80" s="11" t="s">
-        <v>251</v>
-      </c>
-      <c r="M80" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="81" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E80" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="81" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
       <c r="E81" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="82" spans="2:13" x14ac:dyDescent="0.25">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="82" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
-      <c r="E82" s="1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="83" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E82" s="1"/>
+      <c r="F82" t="s">
+        <v>6</v>
+      </c>
+      <c r="H82" t="s">
+        <v>186</v>
+      </c>
+      <c r="I82" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J82" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K82" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="M82" t="s">
+        <v>300</v>
+      </c>
+      <c r="N82" t="s">
+        <v>298</v>
+      </c>
+      <c r="O82" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="83" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
       <c r="E83" s="1"/>
       <c r="F83" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H83" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I83" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K83" s="8" t="s">
-        <v>157</v>
+        <v>2</v>
       </c>
       <c r="M83" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="84" spans="2:13" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+      <c r="N83" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="84" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
       <c r="E84" s="1"/>
       <c r="F84" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="H84" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I84" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="K84" s="8" t="s">
+        <v>189</v>
       </c>
       <c r="M84" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="85" spans="2:13" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+      <c r="N84" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="85" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
       <c r="E85" s="1"/>
       <c r="F85" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H85" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I85" s="3" t="s">
         <v>127</v>
@@ -2674,45 +2789,42 @@
         <v>4</v>
       </c>
       <c r="K85" s="8" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="M85" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="86" spans="2:13" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="86" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
       <c r="E86" s="1"/>
       <c r="F86" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H86" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="I86" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K86" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="L86" s="11" t="s">
-        <v>269</v>
+        <v>193</v>
+      </c>
+      <c r="L86" s="10" t="s">
+        <v>260</v>
       </c>
       <c r="M86" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="87" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
       <c r="E87" s="1"/>
-      <c r="F87" t="s">
-        <v>52</v>
-      </c>
-      <c r="H87" t="s">
-        <v>192</v>
+      <c r="F87" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="I87" s="3" t="s">
         <v>135</v>
@@ -2720,41 +2832,36 @@
       <c r="J87" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="K87" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="L87" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="M87" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="88" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="L87" s="10" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="88" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
       <c r="E88" s="1"/>
-      <c r="F88" s="1" t="s">
-        <v>114</v>
+      <c r="F88" s="1"/>
+      <c r="G88" t="s">
+        <v>53</v>
+      </c>
+      <c r="H88" t="s">
+        <v>194</v>
       </c>
       <c r="I88" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L88" s="11" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="89" spans="2:13" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="89" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
       <c r="E89" s="1"/>
       <c r="F89" s="1"/>
       <c r="G89" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H89" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I89" s="3" t="s">
         <v>127</v>
@@ -2762,74 +2869,70 @@
       <c r="J89" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="L89" s="11"/>
-    </row>
-    <row r="90" spans="2:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
       <c r="E90" s="1"/>
       <c r="F90" s="1"/>
       <c r="G90" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H90" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I90" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J90" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="L90" s="11"/>
-    </row>
-    <row r="91" spans="2:13" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
       <c r="E91" s="1"/>
-      <c r="F91" s="1"/>
-      <c r="G91" t="s">
-        <v>55</v>
-      </c>
-      <c r="H91" t="s">
-        <v>196</v>
-      </c>
-      <c r="I91" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J91" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="L91" s="11"/>
-    </row>
-    <row r="92" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="F91" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="92" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
-      <c r="E92" s="1"/>
-      <c r="F92" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="93" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E92" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="93" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
       <c r="E93" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="94" spans="2:13" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="94" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
-      <c r="E94" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="L94" s="10" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="95" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E94" s="1"/>
+      <c r="F94" t="s">
+        <v>58</v>
+      </c>
+      <c r="H94" t="s">
+        <v>181</v>
+      </c>
+      <c r="I94" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J94" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="M94" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="95" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
       <c r="E95" s="1"/>
       <c r="F95" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H95" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I95" s="3" t="s">
         <v>127</v>
@@ -2837,125 +2940,136 @@
       <c r="J95" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="K95" s="8" t="s">
+        <v>183</v>
+      </c>
       <c r="M95" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="96" spans="2:13" x14ac:dyDescent="0.25">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="96" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
-      <c r="E96" s="1"/>
-      <c r="F96" t="s">
-        <v>59</v>
-      </c>
-      <c r="H96" t="s">
-        <v>182</v>
-      </c>
-      <c r="I96" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J96" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K96" s="8" t="s">
-        <v>183</v>
-      </c>
-      <c r="M96" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="97" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E96" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
-      <c r="E97" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="98" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D97" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="98" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
       <c r="D98" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="99" spans="2:13" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="99" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
-      <c r="D99" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="100" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D99" s="1"/>
+      <c r="E99" t="s">
+        <v>7</v>
+      </c>
+      <c r="H99" t="s">
+        <v>197</v>
+      </c>
+      <c r="I99" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J99" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K99" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="L99" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="M99" t="s">
+        <v>297</v>
+      </c>
+      <c r="N99" t="s">
+        <v>296</v>
+      </c>
+      <c r="O99" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="100" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
-      <c r="D100" s="1"/>
-      <c r="E100" t="s">
-        <v>7</v>
-      </c>
-      <c r="H100" t="s">
-        <v>197</v>
-      </c>
-      <c r="I100" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J100" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K100" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="L100" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="M100" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="101" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D100" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="101" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
       <c r="D101" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="102" spans="2:13" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="102" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
-      <c r="D102" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="103" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D102" s="1"/>
+      <c r="E102" t="s">
+        <v>7</v>
+      </c>
+      <c r="H102" t="s">
+        <v>199</v>
+      </c>
+      <c r="I102" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J102" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K102" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="L102" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="M102" t="s">
+        <v>297</v>
+      </c>
+      <c r="N102" t="s">
+        <v>296</v>
+      </c>
+      <c r="O102" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="103" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
-      <c r="D103" s="1"/>
-      <c r="E103" t="s">
-        <v>7</v>
-      </c>
-      <c r="H103" t="s">
-        <v>199</v>
-      </c>
-      <c r="I103" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J103" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K103" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="L103" s="10" t="s">
-        <v>277</v>
-      </c>
-      <c r="M103" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="104" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D103" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="104" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
       <c r="D104" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="105" spans="2:13" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+      <c r="H104" t="s">
+        <v>201</v>
+      </c>
+      <c r="I104" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J104" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M104" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="105" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
-      <c r="D105" s="1" t="s">
-        <v>118</v>
+      <c r="E105" t="s">
+        <v>64</v>
       </c>
       <c r="H105" t="s">
-        <v>201</v>
+        <v>184</v>
       </c>
       <c r="I105" s="3" t="s">
         <v>135</v>
@@ -2963,32 +3077,32 @@
       <c r="J105" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M105" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="106" spans="2:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
       <c r="E106" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="H106" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="I106" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J106" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="107" spans="2:13" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="K106" s="8" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="107" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
       <c r="E107" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="H107" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="I107" s="3" t="s">
         <v>127</v>
@@ -2997,58 +3111,61 @@
         <v>4</v>
       </c>
       <c r="K107" s="8" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="108" spans="2:13" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+      <c r="L107" s="10" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="108" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
       <c r="E108" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H108" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="I108" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J108" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K108" s="8" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="109" spans="2:13" x14ac:dyDescent="0.25">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="109" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
-      <c r="E109" t="s">
-        <v>66</v>
-      </c>
-      <c r="H109" t="s">
-        <v>203</v>
-      </c>
-      <c r="I109" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J109" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K109" s="8" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="110" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D109" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="110" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
       <c r="D110" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="111" spans="2:13" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+      <c r="H110" t="s">
+        <v>207</v>
+      </c>
+      <c r="I110" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J110" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M110" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="111" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
-      <c r="D111" s="1" t="s">
-        <v>119</v>
+      <c r="E111" t="s">
+        <v>64</v>
       </c>
       <c r="H111" t="s">
-        <v>207</v>
+        <v>184</v>
       </c>
       <c r="I111" s="3" t="s">
         <v>135</v>
@@ -3057,31 +3174,43 @@
         <v>2</v>
       </c>
       <c r="M111" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="112" spans="2:13" x14ac:dyDescent="0.25">
+        <v>307</v>
+      </c>
+      <c r="N111" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="112" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
       <c r="E112" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="H112" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
       <c r="I112" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J112" s="4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="113" spans="2:13" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="K112" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="M112" t="s">
+        <v>307</v>
+      </c>
+      <c r="N112" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="113" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
       <c r="E113" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="H113" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="I113" s="3" t="s">
         <v>127</v>
@@ -3090,64 +3219,73 @@
         <v>4</v>
       </c>
       <c r="K113" s="8" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="114" spans="2:13" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+      <c r="L113" s="10" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="114" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
       <c r="E114" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H114" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="I114" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J114" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K114" s="8" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="115" spans="2:13" x14ac:dyDescent="0.25">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="115" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
-      <c r="E115" t="s">
-        <v>66</v>
-      </c>
-      <c r="H115" t="s">
-        <v>203</v>
-      </c>
-      <c r="I115" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J115" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K115" s="8" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="116" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D115" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="116" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
       <c r="D116" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="117" spans="2:13" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="117" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
-      <c r="D117" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="118" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E117" t="s">
+        <v>69</v>
+      </c>
+      <c r="H117" t="s">
+        <v>208</v>
+      </c>
+      <c r="I117" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J117" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L117" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="M117" t="s">
+        <v>312</v>
+      </c>
+      <c r="N117" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="118" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
       <c r="E118" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H118" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I118" s="3" t="s">
         <v>127</v>
@@ -3155,95 +3293,113 @@
       <c r="J118" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="K118" s="8" t="s">
+        <v>210</v>
+      </c>
       <c r="L118" s="10" t="s">
-        <v>266</v>
+        <v>313</v>
       </c>
       <c r="M118" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="119" spans="2:13" x14ac:dyDescent="0.25">
+        <v>312</v>
+      </c>
+      <c r="N118" t="s">
+        <v>270</v>
+      </c>
+      <c r="O118" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="119" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
-      <c r="E119" t="s">
-        <v>70</v>
-      </c>
-      <c r="H119" t="s">
-        <v>209</v>
-      </c>
-      <c r="I119" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J119" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K119" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="M119" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="120" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D119" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="120" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
       <c r="D120" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="121" spans="2:13" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="121" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
-      <c r="D121" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="122" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E121" t="s">
+        <v>72</v>
+      </c>
+      <c r="H121" t="s">
+        <v>211</v>
+      </c>
+      <c r="I121" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J121" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K121" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="L121" s="10" t="s">
+        <v>249</v>
+      </c>
+      <c r="M121" t="s">
+        <v>319</v>
+      </c>
+      <c r="N121" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="122" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
       <c r="E122" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H122" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I122" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J122" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K122" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="L122" s="10" t="s">
-        <v>254</v>
+        <v>4</v>
       </c>
       <c r="M122" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="123" spans="2:13" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="N122" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="123" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
       <c r="E123" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H123" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I123" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J123" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="K123" s="8" t="s">
+        <v>214</v>
       </c>
       <c r="M123" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="124" spans="2:13" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="N123" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="124" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
       <c r="E124" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H124" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I124" s="3" t="s">
         <v>135</v>
@@ -3251,84 +3407,96 @@
       <c r="J124" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="K124" s="8" t="s">
-        <v>214</v>
-      </c>
       <c r="M124" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="125" spans="2:13" x14ac:dyDescent="0.25">
+        <v>319</v>
+      </c>
+      <c r="N124" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="125" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
-      <c r="E125" t="s">
-        <v>75</v>
-      </c>
-      <c r="H125" t="s">
-        <v>215</v>
-      </c>
-      <c r="I125" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J125" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="M125" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="126" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D125" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="126" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
       <c r="D126" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="127" spans="2:13" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="127" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
-      <c r="D127" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="128" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D127" s="1"/>
+      <c r="E127" t="s">
+        <v>77</v>
+      </c>
+      <c r="H127" t="s">
+        <v>217</v>
+      </c>
+      <c r="I127" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J127" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K127" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="M127" t="s">
+        <v>272</v>
+      </c>
+      <c r="N127" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="128" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
-      <c r="D128" s="1"/>
-      <c r="E128" t="s">
-        <v>77</v>
-      </c>
-      <c r="H128" t="s">
-        <v>217</v>
-      </c>
-      <c r="I128" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J128" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K128" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="M128" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="129" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D128" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="129" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
       <c r="D129" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="130" spans="2:13" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="130" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
-      <c r="D130" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="131" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E130" t="s">
+        <v>6</v>
+      </c>
+      <c r="H130" t="s">
+        <v>219</v>
+      </c>
+      <c r="I130" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J130" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="M130" t="s">
+        <v>270</v>
+      </c>
+      <c r="N130" t="s">
+        <v>320</v>
+      </c>
+      <c r="O130" t="s">
+        <v>321</v>
+      </c>
+      <c r="P130" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="131" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
       <c r="E131" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
       <c r="H131" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I131" s="3" t="s">
         <v>127</v>
@@ -3337,250 +3505,296 @@
         <v>4</v>
       </c>
       <c r="M131" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="132" spans="2:13" x14ac:dyDescent="0.25">
+        <v>270</v>
+      </c>
+      <c r="N131" t="s">
+        <v>320</v>
+      </c>
+      <c r="O131" t="s">
+        <v>321</v>
+      </c>
+      <c r="P131" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="132" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
       <c r="E132" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H132" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I132" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J132" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="K132" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="L132" s="10" t="s">
+        <v>252</v>
       </c>
       <c r="M132" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="133" spans="2:13" x14ac:dyDescent="0.25">
+        <v>270</v>
+      </c>
+      <c r="N132" t="s">
+        <v>320</v>
+      </c>
+      <c r="O132" t="s">
+        <v>321</v>
+      </c>
+      <c r="P132" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="133" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
       <c r="E133" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H133" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="I133" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J133" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K133" s="8" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="L133" s="10" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="M133" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="134" spans="2:13" x14ac:dyDescent="0.25">
+        <v>270</v>
+      </c>
+      <c r="N133" t="s">
+        <v>320</v>
+      </c>
+      <c r="O133" t="s">
+        <v>321</v>
+      </c>
+      <c r="P133" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="134" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
-      <c r="E134" t="s">
-        <v>81</v>
-      </c>
-      <c r="H134" t="s">
-        <v>223</v>
-      </c>
-      <c r="I134" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J134" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K134" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="L134" s="10" t="s">
-        <v>256</v>
-      </c>
-      <c r="M134" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="135" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E134" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="135" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
-      <c r="E135" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="136" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E135" s="1"/>
+      <c r="F135" t="s">
+        <v>64</v>
+      </c>
+      <c r="H135" t="s">
+        <v>224</v>
+      </c>
+      <c r="I135" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J135" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="K135" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="M135" t="s">
+        <v>270</v>
+      </c>
+      <c r="N135" t="s">
+        <v>320</v>
+      </c>
+      <c r="O135" t="s">
+        <v>321</v>
+      </c>
+      <c r="P135" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="136" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
-      <c r="E136" s="1"/>
-      <c r="F136" t="s">
-        <v>64</v>
-      </c>
-      <c r="H136" t="s">
-        <v>224</v>
-      </c>
-      <c r="I136" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J136" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K136" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="M136" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="137" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E136" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="137" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
-      <c r="E137" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="138" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D137" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="138" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
       <c r="D138" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="139" spans="2:13" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="139" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
-      <c r="D139" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="140" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="D139" s="1"/>
+      <c r="E139" t="s">
+        <v>6</v>
+      </c>
+      <c r="H139" t="s">
+        <v>227</v>
+      </c>
+      <c r="I139" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J139" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L139" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="M139" t="s">
+        <v>270</v>
+      </c>
+      <c r="N139" t="s">
+        <v>320</v>
+      </c>
+      <c r="O139" t="s">
+        <v>321</v>
+      </c>
+      <c r="P139" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="140" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
       <c r="D140" s="1"/>
       <c r="E140" t="s">
-        <v>6</v>
+        <v>80</v>
       </c>
       <c r="H140" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="I140" s="3" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J140" s="4" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L140" s="11" t="s">
-        <v>258</v>
+        <v>330</v>
       </c>
       <c r="M140" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="141" spans="2:13" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="141" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
       <c r="D141" s="1"/>
       <c r="E141" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H141" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="I141" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J141" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="K141" s="8" t="s">
+        <v>225</v>
       </c>
       <c r="L141" s="11"/>
       <c r="M141" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="142" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
       <c r="D142" s="1"/>
-      <c r="E142" t="s">
-        <v>81</v>
-      </c>
-      <c r="H142" t="s">
-        <v>223</v>
-      </c>
-      <c r="I142" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J142" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K142" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="L142" s="11"/>
-      <c r="M142" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="143" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E142" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="143" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
       <c r="D143" s="1"/>
-      <c r="E143" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="144" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="E143" s="1"/>
+      <c r="F143" t="s">
+        <v>64</v>
+      </c>
+      <c r="H143" t="s">
+        <v>229</v>
+      </c>
+      <c r="I143" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J143" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K143" s="8" t="s">
+        <v>226</v>
+      </c>
+      <c r="L143" s="11"/>
+    </row>
+    <row r="144" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
       <c r="D144" s="1"/>
-      <c r="E144" s="1"/>
-      <c r="F144" t="s">
-        <v>64</v>
-      </c>
-      <c r="H144" t="s">
-        <v>229</v>
-      </c>
-      <c r="I144" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="J144" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="K144" s="8" t="s">
-        <v>226</v>
-      </c>
-      <c r="L144" s="11"/>
-    </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E144" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
-      <c r="D145" s="1"/>
-      <c r="E145" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D145" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
       <c r="D146" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+      <c r="H146" t="s">
+        <v>254</v>
+      </c>
+      <c r="L146" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="M146" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
-      <c r="D147" s="1" t="s">
-        <v>126</v>
+      <c r="D147" s="1"/>
+      <c r="E147" t="s">
+        <v>20</v>
       </c>
       <c r="H147" t="s">
-        <v>259</v>
-      </c>
-      <c r="L147" s="11" t="s">
-        <v>260</v>
-      </c>
-      <c r="M147" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+      <c r="I147" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J147" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="L147" s="13"/>
+    </row>
+    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
       <c r="D148" s="1"/>
       <c r="E148" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H148" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I148" s="3" t="s">
         <v>135</v>
@@ -3588,41 +3802,45 @@
       <c r="J148" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L148" s="11" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K148" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="L148" s="13"/>
+      <c r="M148" t="s">
+        <v>328</v>
+      </c>
+      <c r="N148" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
       <c r="D149" s="1"/>
       <c r="E149" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H149" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="I149" s="3" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="J149" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K149" s="8" t="s">
-        <v>231</v>
-      </c>
-      <c r="L149" s="11"/>
-      <c r="M149" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+      <c r="L149" s="13"/>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
       <c r="D150" s="1"/>
       <c r="E150" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H150" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I150" s="3" t="s">
         <v>127</v>
@@ -3633,16 +3851,16 @@
       <c r="K150" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="L150" s="11"/>
-    </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="L150" s="13"/>
+    </row>
+    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
       <c r="D151" s="1"/>
       <c r="E151" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H151" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I151" s="3" t="s">
         <v>127</v>
@@ -3651,46 +3869,52 @@
         <v>4</v>
       </c>
       <c r="K151" s="8" t="s">
-        <v>230</v>
-      </c>
-      <c r="L151" s="11"/>
-    </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+      <c r="L151" s="13"/>
+    </row>
+    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
       <c r="D152" s="1"/>
-      <c r="E152" t="s">
-        <v>25</v>
-      </c>
-      <c r="H152" t="s">
-        <v>150</v>
-      </c>
-      <c r="I152" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J152" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K152" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="L152" s="11"/>
-    </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E152" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
       <c r="D153" s="1"/>
-      <c r="E153" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E153" s="1"/>
+      <c r="F153" t="s">
+        <v>6</v>
+      </c>
+      <c r="H153" t="s">
+        <v>232</v>
+      </c>
+      <c r="I153" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J153" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="L153" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="M153" t="s">
+        <v>272</v>
+      </c>
+      <c r="N153" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
       <c r="D154" s="1"/>
       <c r="E154" s="1"/>
       <c r="F154" t="s">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="H154" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="I154" s="3" t="s">
         <v>127</v>
@@ -3698,70 +3922,47 @@
       <c r="J154" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="K154" s="8" t="s">
+        <v>234</v>
+      </c>
       <c r="L154" s="10" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="M154" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
       <c r="D155" s="1"/>
-      <c r="E155" s="1"/>
-      <c r="F155" t="s">
-        <v>85</v>
-      </c>
-      <c r="H155" t="s">
-        <v>233</v>
-      </c>
-      <c r="I155" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J155" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K155" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="L155" s="10" t="s">
-        <v>265</v>
-      </c>
-      <c r="M155" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="E155" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
-      <c r="D156" s="1"/>
-      <c r="E156" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D156" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
-      <c r="D157" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B158" s="1"/>
-      <c r="C158" s="1" t="s">
+      <c r="C157" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B159" s="1" t="s">
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B158" s="1" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A159" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A161" s="1" t="s">
         <v>90</v>
       </c>
     </row>

</xml_diff>